<commit_message>
WIP: support for Init Failed reports
</commit_message>
<xml_diff>
--- a/Docs/2020-11-18/ProposedFailedInit-pmk.xlsx
+++ b/Docs/2020-11-18/ProposedFailedInit-pmk.xlsx
@@ -1,16 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://datasages-my.sharepoint.com/personal/pete_datasages_com/Documents/Client Projects/Collins Aerospace/Railwaynet/STROLR Upgrade/Amtrak Reporting/Message Formats from Deji/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="8_{2D81AB3D-C30F-9843-951C-C00C7584294D}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{3C1DC25E-786C-0045-B1FC-590BF444C19A}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="7" rupBuild="9303"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="57400" yWindow="9340" windowWidth="27240" windowHeight="16440" xr2:uid="{2A9EFAF0-DB99-3340-BD9D-5ACF0FB3E174}"/>
+    <workbookView xWindow="57398" yWindow="9338" windowWidth="19395" windowHeight="10995"/>
   </bookViews>
   <sheets>
     <sheet name="Failed Initializations.L" sheetId="1" r:id="rId1"/>
@@ -105,7 +99,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -164,10 +158,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -476,48 +470,48 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B6F7C03-5E8E-0347-A329-48668A6C6A70}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="42.33203125" customWidth="1"/>
-    <col min="2" max="2" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="42.3125" customWidth="1"/>
+    <col min="2" max="2" width="16.6875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.6875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="21.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.6875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.6875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.6875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.1875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="26.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="26.3125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="6" t="s">
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="I1" s="6"/>
+      <c r="I1" s="7"/>
       <c r="J1" s="4"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -549,7 +543,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -581,7 +575,7 @@
         <v>1005</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A4" t="s">
         <v>18</v>
       </c>

</xml_diff>